<commit_message>
update relation type 5a427158f3fac8d86d06da6ea2ad276d7628099c
</commit_message>
<xml_diff>
--- a/ig/nr-update-relationship/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-update-relationship/StructureDefinition-fr-core-patient-ins.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-18T12:45:56+00:00</t>
+    <t>2024-03-22T10:23:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2275,28 +2275,28 @@
     <t>NK1-7, NK1-3</t>
   </si>
   <si>
-    <t>Patient.contact.relationship:RolePerson</t>
-  </si>
-  <si>
-    <t>RolePerson</t>
+    <t>Patient.contact.relationship:Role</t>
+  </si>
+  <si>
+    <t>Role</t>
   </si>
   <si>
     <t>The nature of the relationship. Rôle de la personne. Ex : personne de confiance, aidant ...</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-related-person-role</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson</t>
-  </si>
-  <si>
-    <t>RelatedPerson</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-patient-contact-role</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:RelationType</t>
+  </si>
+  <si>
+    <t>RelationType</t>
   </si>
   <si>
     <t>The nature of the relationship. Relation de la personne. Ex : Mère, époux, enfant ...</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-related-person</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-relation-type</t>
   </si>
   <si>
     <t>Patient.contact.name</t>
@@ -2935,7 +2935,7 @@
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="59.546875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="60.12109375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="75.2109375" customWidth="true" bestFit="true"/>

</xml_diff>